<commit_message>
v3.4.1: catalyst gate + market scanner, one ORB trigger, simplified risk, IST timestamps, continuous news ingestion, Railway self-heal
</commit_message>
<xml_diff>
--- a/Masterdata/master_database.xlsx
+++ b/Masterdata/master_database.xlsx
@@ -3323,7 +3323,7 @@
       <c r="N45" s="2" t="n"/>
       <c r="O45" s="2" t="inlineStr">
         <is>
-          <t>BATTERIES | AUTO | INDUSTRIAL</t>
+          <t>BATTERIES | INDUSTRIAL</t>
         </is>
       </c>
       <c r="P45" s="2" t="inlineStr">
@@ -7563,7 +7563,7 @@
       <c r="N109" s="2" t="n"/>
       <c r="O109" s="2" t="inlineStr">
         <is>
-          <t>FORGINGS | AUTO | INDUSTRIAL</t>
+          <t>FORGINGS | INDUSTRIAL</t>
         </is>
       </c>
       <c r="P109" s="2" t="inlineStr">
@@ -15533,7 +15533,7 @@
       <c r="N230" s="2" t="n"/>
       <c r="O230" s="2" t="inlineStr">
         <is>
-          <t>BATTERIES | AUTO | INDUSTRIAL</t>
+          <t>BATTERIES | INDUSTRIAL</t>
         </is>
       </c>
       <c r="P230" s="2" t="inlineStr">
@@ -40201,7 +40201,7 @@
       <c r="N604" s="2" t="n"/>
       <c r="O604" s="2" t="inlineStr">
         <is>
-          <t>POWER EQUIPMENT | ENERGY</t>
+          <t>POWER EQUIPMENT</t>
         </is>
       </c>
       <c r="P604" s="2" t="inlineStr">
@@ -40267,7 +40267,7 @@
       <c r="N605" s="2" t="n"/>
       <c r="O605" s="2" t="inlineStr">
         <is>
-          <t>INDUSTRIAL AUTOMATION | ENERGY | MOBILITY</t>
+          <t>INDUSTRIAL AUTOMATION | MOBILITY</t>
         </is>
       </c>
       <c r="P605" s="2" t="inlineStr">
@@ -42707,11 +42707,7 @@
       <c r="L642" s="2" t="n"/>
       <c r="M642" s="2" t="n"/>
       <c r="N642" s="2" t="n"/>
-      <c r="O642" s="2" t="inlineStr">
-        <is>
-          <t>ENERGY</t>
-        </is>
-      </c>
+      <c r="O642" s="2" t="inlineStr"/>
       <c r="P642" s="2" t="inlineStr">
         <is>
           <t>EPC | CONSTRUCTION | ENERGY | INFRASTRUCTURE</t>

</xml_diff>